<commit_message>
Finish native visual review and preserve scoped evidence context
</commit_message>
<xml_diff>
--- a/docs/legal/gap-instruments/evidence-tracking/tracker.xlsx
+++ b/docs/legal/gap-instruments/evidence-tracking/tracker.xlsx
@@ -290,7 +290,7 @@
     <t>State SHA-256</t>
   </si>
   <si>
-    <t>dde6c0ebd5e7d1d19757346feade554732bcb34ce35e90f8ab7e5101923021f9</t>
+    <t>a31397f46b49101ba75d632de23edbfc8eef3205c77571e41fe653be2fa8def5</t>
   </si>
   <si>
     <t>docs/finance/evidence/SH-FIN-HUMAN-001/source.json</t>
@@ -302,7 +302,7 @@
     <t>docs/legal/gap-instruments/period-close/README.md</t>
   </si>
   <si>
-    <t>1f764afff496bd216dfca3fd1ffac4accf7433cf0404557f894312f82887577a</t>
+    <t>2cf05a38cb0a634ba8355e6f5e046977ada35dad0a83d210b7cd265491c59e20</t>
   </si>
   <si>
     <t>docs/legal/gap-instruments/period-close/case.json</t>

</xml_diff>